<commit_message>
include size 46 in EB Shoes size column mapping
</commit_message>
<xml_diff>
--- a/po_template/PO TK TEMPLATE.xlsx
+++ b/po_template/PO TK TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EVERBEST\NEW_GENERATOR\webapp\po_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16423A40-2D90-4DFA-917F-C17878F82142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE47AB42-553D-4BF4-9EFF-B9DE3D7A7AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PO" sheetId="4" r:id="rId1"/>
@@ -2210,219 +2210,6 @@
     <xf numFmtId="165" fontId="13" fillId="7" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="50" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="52" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="40" fillId="5" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="40" fillId="5" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="40" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="40" fillId="5" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="49" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="51" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="53" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2522,6 +2309,9 @@
     <xf numFmtId="0" fontId="34" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2529,6 +2319,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2541,8 +2334,215 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="49" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="51" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="53" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="50" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="52" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="40" fillId="5" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="40" fillId="5" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="40" fillId="5" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="40" fillId="5" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="29" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -3309,7 +3309,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>628650</xdr:colOff>
+      <xdr:colOff>507054</xdr:colOff>
       <xdr:row>47</xdr:row>
       <xdr:rowOff>73602</xdr:rowOff>
     </xdr:to>
@@ -4430,7 +4430,8 @@
     <col min="4" max="4" width="24.85546875" style="26" customWidth="1"/>
     <col min="5" max="5" width="20" style="25" customWidth="1"/>
     <col min="6" max="8" width="10" style="25" customWidth="1"/>
-    <col min="9" max="18" width="7.5703125" style="25" customWidth="1"/>
+    <col min="9" max="17" width="7.5703125" style="25" customWidth="1"/>
+    <col min="18" max="18" width="9.28515625" style="25" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="15.5703125" style="25" customWidth="1"/>
     <col min="20" max="20" width="12.28515625" style="27" customWidth="1"/>
     <col min="21" max="21" width="20.28515625" style="28" customWidth="1"/>
@@ -4439,11 +4440,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="23.25">
-      <c r="A1" s="149" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="149"/>
-      <c r="C1" s="149"/>
+      <c r="A1" s="244" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="244"/>
+      <c r="C1" s="244"/>
       <c r="D1" s="30"/>
       <c r="E1" s="31"/>
       <c r="F1" s="31"/>
@@ -4451,14 +4452,14 @@
       <c r="H1" s="31"/>
       <c r="I1" s="30"/>
       <c r="J1" s="30"/>
-      <c r="N1" s="150"/>
-      <c r="O1" s="150"/>
-      <c r="P1" s="150"/>
-      <c r="Q1" s="150"/>
-      <c r="R1" s="150"/>
-      <c r="S1" s="150"/>
-      <c r="T1" s="150"/>
-      <c r="U1" s="150"/>
+      <c r="N1" s="245"/>
+      <c r="O1" s="245"/>
+      <c r="P1" s="245"/>
+      <c r="Q1" s="245"/>
+      <c r="R1" s="245"/>
+      <c r="S1" s="245"/>
+      <c r="T1" s="245"/>
+      <c r="U1" s="245"/>
     </row>
     <row r="2" spans="1:22" ht="23.25" customHeight="1">
       <c r="A2" s="32" t="s">
@@ -4469,47 +4470,47 @@
       </c>
       <c r="C2" s="34"/>
       <c r="D2" s="35"/>
-      <c r="E2" s="151" t="s">
+      <c r="E2" s="246" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="151"/>
-      <c r="G2" s="151"/>
-      <c r="H2" s="151"/>
-      <c r="I2" s="151"/>
-      <c r="J2" s="151"/>
-      <c r="K2" s="151"/>
-      <c r="N2" s="152" t="s">
+      <c r="F2" s="246"/>
+      <c r="G2" s="246"/>
+      <c r="H2" s="246"/>
+      <c r="I2" s="246"/>
+      <c r="J2" s="246"/>
+      <c r="K2" s="246"/>
+      <c r="N2" s="247" t="s">
         <v>3</v>
       </c>
-      <c r="O2" s="152"/>
-      <c r="P2" s="152"/>
-      <c r="Q2" s="152"/>
-      <c r="R2" s="152"/>
-      <c r="S2" s="152"/>
-      <c r="T2" s="152"/>
-      <c r="U2" s="152"/>
+      <c r="O2" s="247"/>
+      <c r="P2" s="247"/>
+      <c r="Q2" s="247"/>
+      <c r="R2" s="247"/>
+      <c r="S2" s="247"/>
+      <c r="T2" s="247"/>
+      <c r="U2" s="247"/>
     </row>
     <row r="3" spans="1:22" ht="21.75" customHeight="1">
       <c r="A3" s="36"/>
       <c r="B3" s="37"/>
       <c r="C3" s="38"/>
-      <c r="E3" s="143"/>
-      <c r="F3" s="143"/>
-      <c r="G3" s="143"/>
-      <c r="H3" s="143"/>
-      <c r="I3" s="143"/>
-      <c r="J3" s="143"/>
-      <c r="K3" s="143"/>
-      <c r="N3" s="153" t="s">
+      <c r="E3" s="248"/>
+      <c r="F3" s="248"/>
+      <c r="G3" s="248"/>
+      <c r="H3" s="248"/>
+      <c r="I3" s="248"/>
+      <c r="J3" s="248"/>
+      <c r="K3" s="248"/>
+      <c r="N3" s="249" t="s">
         <v>4</v>
       </c>
-      <c r="O3" s="153"/>
-      <c r="P3" s="153"/>
-      <c r="Q3" s="153"/>
-      <c r="R3" s="153"/>
-      <c r="S3" s="153"/>
-      <c r="T3" s="153"/>
-      <c r="U3" s="153"/>
+      <c r="O3" s="249"/>
+      <c r="P3" s="249"/>
+      <c r="Q3" s="249"/>
+      <c r="R3" s="249"/>
+      <c r="S3" s="249"/>
+      <c r="T3" s="249"/>
+      <c r="U3" s="249"/>
     </row>
     <row r="4" spans="1:22" ht="21.75" customHeight="1">
       <c r="A4" s="36" t="s">
@@ -4517,193 +4518,193 @@
       </c>
       <c r="B4" s="37"/>
       <c r="C4" s="39"/>
-      <c r="E4" s="143"/>
-      <c r="F4" s="143"/>
-      <c r="G4" s="143"/>
-      <c r="H4" s="143"/>
-      <c r="I4" s="143"/>
-      <c r="J4" s="143"/>
-      <c r="K4" s="143"/>
-      <c r="N4" s="144" t="s">
+      <c r="E4" s="248"/>
+      <c r="F4" s="248"/>
+      <c r="G4" s="248"/>
+      <c r="H4" s="248"/>
+      <c r="I4" s="248"/>
+      <c r="J4" s="248"/>
+      <c r="K4" s="248"/>
+      <c r="N4" s="250" t="s">
         <v>6</v>
       </c>
-      <c r="O4" s="144"/>
-      <c r="P4" s="144"/>
-      <c r="Q4" s="144"/>
-      <c r="R4" s="144"/>
-      <c r="S4" s="144"/>
-      <c r="T4" s="144"/>
-      <c r="U4" s="144"/>
+      <c r="O4" s="250"/>
+      <c r="P4" s="250"/>
+      <c r="Q4" s="250"/>
+      <c r="R4" s="250"/>
+      <c r="S4" s="250"/>
+      <c r="T4" s="250"/>
+      <c r="U4" s="250"/>
     </row>
     <row r="5" spans="1:22" ht="21.75" customHeight="1">
       <c r="A5" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="145" t="s">
+      <c r="B5" s="251" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="146"/>
+      <c r="C5" s="252"/>
       <c r="D5" s="41"/>
-      <c r="E5" s="143"/>
-      <c r="F5" s="143"/>
-      <c r="G5" s="143"/>
-      <c r="H5" s="143"/>
-      <c r="I5" s="143"/>
-      <c r="J5" s="143"/>
-      <c r="K5" s="143"/>
-      <c r="N5" s="144" t="s">
+      <c r="E5" s="248"/>
+      <c r="F5" s="248"/>
+      <c r="G5" s="248"/>
+      <c r="H5" s="248"/>
+      <c r="I5" s="248"/>
+      <c r="J5" s="248"/>
+      <c r="K5" s="248"/>
+      <c r="N5" s="250" t="s">
         <v>71</v>
       </c>
-      <c r="O5" s="144"/>
-      <c r="P5" s="144"/>
-      <c r="Q5" s="144"/>
-      <c r="R5" s="144"/>
-      <c r="S5" s="144"/>
-      <c r="T5" s="144"/>
-      <c r="U5" s="144"/>
+      <c r="O5" s="250"/>
+      <c r="P5" s="250"/>
+      <c r="Q5" s="250"/>
+      <c r="R5" s="250"/>
+      <c r="S5" s="250"/>
+      <c r="T5" s="250"/>
+      <c r="U5" s="250"/>
     </row>
     <row r="6" spans="1:22" ht="21.75" customHeight="1">
       <c r="A6" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="147" t="s">
+      <c r="B6" s="253" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="148"/>
+      <c r="C6" s="254"/>
       <c r="D6" s="41"/>
-      <c r="N6" s="144"/>
-      <c r="O6" s="144"/>
-      <c r="P6" s="144"/>
-      <c r="Q6" s="144"/>
-      <c r="R6" s="144"/>
-      <c r="S6" s="144"/>
+      <c r="N6" s="250"/>
+      <c r="O6" s="250"/>
+      <c r="P6" s="250"/>
+      <c r="Q6" s="250"/>
+      <c r="R6" s="250"/>
+      <c r="S6" s="250"/>
       <c r="T6" s="92"/>
     </row>
     <row r="8" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A8" s="199" t="s">
+      <c r="A8" s="193" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="190" t="s">
+      <c r="B8" s="242" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="202" t="s">
+      <c r="C8" s="196" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="204" t="s">
+      <c r="D8" s="198" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="206" t="s">
+      <c r="E8" s="201" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="194" t="s">
+      <c r="F8" s="209" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="212"/>
-      <c r="H8" s="212"/>
-      <c r="I8" s="212"/>
-      <c r="J8" s="212"/>
-      <c r="K8" s="212"/>
-      <c r="L8" s="212"/>
-      <c r="M8" s="212"/>
-      <c r="N8" s="212"/>
-      <c r="O8" s="212"/>
-      <c r="P8" s="212"/>
-      <c r="Q8" s="212"/>
-      <c r="R8" s="209" t="s">
+      <c r="G8" s="210"/>
+      <c r="H8" s="210"/>
+      <c r="I8" s="210"/>
+      <c r="J8" s="210"/>
+      <c r="K8" s="210"/>
+      <c r="L8" s="210"/>
+      <c r="M8" s="210"/>
+      <c r="N8" s="210"/>
+      <c r="O8" s="210"/>
+      <c r="P8" s="210"/>
+      <c r="Q8" s="210"/>
+      <c r="R8" s="206" t="s">
         <v>17</v>
       </c>
-      <c r="S8" s="157" t="s">
+      <c r="S8" s="215" t="s">
         <v>18</v>
       </c>
-      <c r="T8" s="159" t="s">
+      <c r="T8" s="217" t="s">
         <v>19</v>
       </c>
       <c r="U8" s="29"/>
       <c r="V8" s="25"/>
     </row>
     <row r="9" spans="1:22" ht="21" customHeight="1">
-      <c r="A9" s="200"/>
-      <c r="B9" s="191"/>
-      <c r="C9" s="203"/>
-      <c r="D9" s="191"/>
-      <c r="E9" s="207"/>
-      <c r="F9" s="192">
+      <c r="A9" s="194"/>
+      <c r="B9" s="199"/>
+      <c r="C9" s="197"/>
+      <c r="D9" s="199"/>
+      <c r="E9" s="202"/>
+      <c r="F9" s="188">
         <f>'packing list'!B7</f>
         <v>26</v>
       </c>
-      <c r="G9" s="192">
+      <c r="G9" s="188">
         <f t="shared" ref="G9:Q9" si="0">F9+1</f>
         <v>27</v>
       </c>
-      <c r="H9" s="192">
+      <c r="H9" s="188">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="I9" s="192">
+      <c r="I9" s="188">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="J9" s="192">
+      <c r="J9" s="188">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="K9" s="192">
+      <c r="K9" s="188">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="L9" s="192">
+      <c r="L9" s="188">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="M9" s="192">
+      <c r="M9" s="188">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="N9" s="192">
+      <c r="N9" s="188">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="O9" s="192">
+      <c r="O9" s="188">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="P9" s="192">
+      <c r="P9" s="188">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="Q9" s="194">
+      <c r="Q9" s="209">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="R9" s="210"/>
-      <c r="S9" s="158"/>
-      <c r="T9" s="160"/>
+      <c r="R9" s="207"/>
+      <c r="S9" s="216"/>
+      <c r="T9" s="218"/>
       <c r="U9" s="29"/>
       <c r="V9" s="25"/>
     </row>
     <row r="10" spans="1:22">
-      <c r="A10" s="201"/>
+      <c r="A10" s="195"/>
       <c r="B10" s="44" t="s">
         <v>20</v>
       </c>
       <c r="C10" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="205"/>
-      <c r="E10" s="208"/>
-      <c r="F10" s="193"/>
-      <c r="G10" s="193"/>
-      <c r="H10" s="193"/>
-      <c r="I10" s="193"/>
-      <c r="J10" s="193"/>
-      <c r="K10" s="193"/>
-      <c r="L10" s="193"/>
-      <c r="M10" s="193"/>
-      <c r="N10" s="193"/>
-      <c r="O10" s="193"/>
-      <c r="P10" s="193"/>
-      <c r="Q10" s="195"/>
-      <c r="R10" s="211"/>
+      <c r="D10" s="200"/>
+      <c r="E10" s="203"/>
+      <c r="F10" s="189"/>
+      <c r="G10" s="189"/>
+      <c r="H10" s="189"/>
+      <c r="I10" s="189"/>
+      <c r="J10" s="189"/>
+      <c r="K10" s="189"/>
+      <c r="L10" s="189"/>
+      <c r="M10" s="189"/>
+      <c r="N10" s="189"/>
+      <c r="O10" s="189"/>
+      <c r="P10" s="189"/>
+      <c r="Q10" s="243"/>
+      <c r="R10" s="208"/>
       <c r="S10" s="113" t="s">
         <v>22</v>
       </c>
@@ -4876,9 +4877,9 @@
       <c r="A17" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="226"/>
-      <c r="C17" s="226"/>
-      <c r="D17" s="227"/>
+      <c r="B17" s="155"/>
+      <c r="C17" s="155"/>
+      <c r="D17" s="156"/>
       <c r="V17" s="129"/>
       <c r="W17" s="130"/>
     </row>
@@ -4886,9 +4887,9 @@
       <c r="A18" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="228"/>
-      <c r="C18" s="228"/>
-      <c r="D18" s="229"/>
+      <c r="B18" s="157"/>
+      <c r="C18" s="157"/>
+      <c r="D18" s="158"/>
       <c r="F18" s="66"/>
       <c r="G18" s="66"/>
       <c r="H18" s="66"/>
@@ -4910,9 +4911,9 @@
       <c r="A19" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="186"/>
-      <c r="C19" s="186"/>
-      <c r="D19" s="187"/>
+      <c r="B19" s="204"/>
+      <c r="C19" s="204"/>
+      <c r="D19" s="205"/>
       <c r="F19" s="66"/>
       <c r="G19" s="66"/>
       <c r="H19" s="66"/>
@@ -4934,9 +4935,9 @@
       <c r="A20" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="188"/>
-      <c r="C20" s="188"/>
-      <c r="D20" s="189"/>
+      <c r="B20" s="240"/>
+      <c r="C20" s="240"/>
+      <c r="D20" s="241"/>
       <c r="F20" s="29"/>
       <c r="G20" s="29"/>
       <c r="H20" s="29"/>
@@ -4960,11 +4961,11 @@
       <c r="A21" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="182" t="s">
+      <c r="B21" s="236" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="182"/>
-      <c r="D21" s="183"/>
+      <c r="C21" s="236"/>
+      <c r="D21" s="237"/>
       <c r="F21" s="29"/>
       <c r="G21" s="29"/>
       <c r="H21" s="29"/>
@@ -4986,9 +4987,9 @@
     </row>
     <row r="22" spans="1:25" ht="24.75" customHeight="1">
       <c r="A22" s="69"/>
-      <c r="B22" s="184"/>
-      <c r="C22" s="184"/>
-      <c r="D22" s="185"/>
+      <c r="B22" s="238"/>
+      <c r="C22" s="238"/>
+      <c r="D22" s="239"/>
       <c r="F22" s="29"/>
       <c r="G22" s="29"/>
       <c r="H22" s="29"/>
@@ -5012,9 +5013,9 @@
       <c r="A23" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="186"/>
-      <c r="C23" s="186"/>
-      <c r="D23" s="187"/>
+      <c r="B23" s="204"/>
+      <c r="C23" s="204"/>
+      <c r="D23" s="205"/>
       <c r="F23" s="29"/>
       <c r="G23" s="29"/>
       <c r="H23" s="29"/>
@@ -5038,11 +5039,11 @@
       <c r="A24" s="71" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="178" t="s">
+      <c r="B24" s="232" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="178"/>
-      <c r="D24" s="179"/>
+      <c r="C24" s="232"/>
+      <c r="D24" s="233"/>
       <c r="F24" s="29"/>
       <c r="G24" s="29"/>
       <c r="H24" s="29"/>
@@ -5064,11 +5065,11 @@
     </row>
     <row r="25" spans="1:25" ht="24.75" customHeight="1" thickBot="1">
       <c r="A25" s="72"/>
-      <c r="B25" s="180"/>
-      <c r="C25" s="180"/>
-      <c r="D25" s="181"/>
-      <c r="I25" s="213"/>
-      <c r="J25" s="213"/>
+      <c r="B25" s="234"/>
+      <c r="C25" s="234"/>
+      <c r="D25" s="235"/>
+      <c r="I25" s="211"/>
+      <c r="J25" s="211"/>
       <c r="V25" s="132"/>
       <c r="W25" s="134"/>
       <c r="X25" s="133"/>
@@ -5091,355 +5092,355 @@
       <c r="W26" s="131"/>
     </row>
     <row r="27" spans="1:25" ht="28.5" customHeight="1">
-      <c r="A27" s="154"/>
-      <c r="B27" s="155"/>
-      <c r="C27" s="155"/>
-      <c r="D27" s="155"/>
-      <c r="E27" s="155"/>
-      <c r="F27" s="155"/>
-      <c r="G27" s="155"/>
-      <c r="H27" s="155"/>
-      <c r="I27" s="155"/>
-      <c r="J27" s="155"/>
-      <c r="K27" s="155"/>
-      <c r="L27" s="155"/>
-      <c r="M27" s="155"/>
-      <c r="N27" s="155"/>
-      <c r="O27" s="155"/>
-      <c r="P27" s="155"/>
-      <c r="Q27" s="155"/>
-      <c r="R27" s="155"/>
-      <c r="S27" s="155"/>
-      <c r="T27" s="155"/>
-      <c r="U27" s="156"/>
+      <c r="A27" s="212"/>
+      <c r="B27" s="213"/>
+      <c r="C27" s="213"/>
+      <c r="D27" s="213"/>
+      <c r="E27" s="213"/>
+      <c r="F27" s="213"/>
+      <c r="G27" s="213"/>
+      <c r="H27" s="213"/>
+      <c r="I27" s="213"/>
+      <c r="J27" s="213"/>
+      <c r="K27" s="213"/>
+      <c r="L27" s="213"/>
+      <c r="M27" s="213"/>
+      <c r="N27" s="213"/>
+      <c r="O27" s="213"/>
+      <c r="P27" s="213"/>
+      <c r="Q27" s="213"/>
+      <c r="R27" s="213"/>
+      <c r="S27" s="213"/>
+      <c r="T27" s="213"/>
+      <c r="U27" s="214"/>
     </row>
     <row r="28" spans="1:25" ht="24.75" customHeight="1">
-      <c r="A28" s="196">
+      <c r="A28" s="190">
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="B28" s="197"/>
-      <c r="C28" s="198"/>
-      <c r="D28" s="197"/>
-      <c r="E28" s="197"/>
-      <c r="F28" s="197"/>
-      <c r="G28" s="197"/>
-      <c r="H28" s="197"/>
-      <c r="I28" s="197"/>
-      <c r="J28" s="197"/>
-      <c r="K28" s="197"/>
-      <c r="L28" s="196" t="s">
+      <c r="B28" s="191"/>
+      <c r="C28" s="192"/>
+      <c r="D28" s="191"/>
+      <c r="E28" s="191"/>
+      <c r="F28" s="191"/>
+      <c r="G28" s="191"/>
+      <c r="H28" s="191"/>
+      <c r="I28" s="191"/>
+      <c r="J28" s="191"/>
+      <c r="K28" s="191"/>
+      <c r="L28" s="190" t="s">
         <v>33</v>
       </c>
-      <c r="M28" s="197"/>
-      <c r="N28" s="197"/>
-      <c r="O28" s="197"/>
-      <c r="P28" s="197"/>
-      <c r="Q28" s="197"/>
-      <c r="R28" s="197"/>
-      <c r="S28" s="197"/>
-      <c r="T28" s="197"/>
-      <c r="U28" s="198"/>
+      <c r="M28" s="191"/>
+      <c r="N28" s="191"/>
+      <c r="O28" s="191"/>
+      <c r="P28" s="191"/>
+      <c r="Q28" s="191"/>
+      <c r="R28" s="191"/>
+      <c r="S28" s="191"/>
+      <c r="T28" s="191"/>
+      <c r="U28" s="192"/>
     </row>
     <row r="29" spans="1:25" ht="24.75" customHeight="1">
-      <c r="A29" s="216"/>
-      <c r="B29" s="216"/>
-      <c r="C29" s="217"/>
-      <c r="D29" s="220"/>
-      <c r="E29" s="221"/>
-      <c r="F29" s="230"/>
-      <c r="G29" s="231"/>
-      <c r="H29" s="231"/>
-      <c r="I29" s="231"/>
-      <c r="J29" s="231"/>
-      <c r="K29" s="232"/>
-      <c r="L29" s="230"/>
-      <c r="M29" s="231"/>
-      <c r="N29" s="231"/>
-      <c r="O29" s="231"/>
-      <c r="P29" s="231"/>
-      <c r="Q29" s="231"/>
-      <c r="R29" s="231"/>
-      <c r="S29" s="231"/>
-      <c r="T29" s="231"/>
-      <c r="U29" s="232"/>
+      <c r="A29" s="145"/>
+      <c r="B29" s="145"/>
+      <c r="C29" s="146"/>
+      <c r="D29" s="149"/>
+      <c r="E29" s="150"/>
+      <c r="F29" s="159"/>
+      <c r="G29" s="160"/>
+      <c r="H29" s="160"/>
+      <c r="I29" s="160"/>
+      <c r="J29" s="160"/>
+      <c r="K29" s="161"/>
+      <c r="L29" s="159"/>
+      <c r="M29" s="160"/>
+      <c r="N29" s="160"/>
+      <c r="O29" s="160"/>
+      <c r="P29" s="160"/>
+      <c r="Q29" s="160"/>
+      <c r="R29" s="160"/>
+      <c r="S29" s="160"/>
+      <c r="T29" s="160"/>
+      <c r="U29" s="161"/>
     </row>
     <row r="30" spans="1:25" ht="24.75" customHeight="1">
-      <c r="A30" s="218"/>
-      <c r="B30" s="218"/>
-      <c r="C30" s="219"/>
-      <c r="D30" s="222"/>
-      <c r="E30" s="223"/>
-      <c r="F30" s="233"/>
-      <c r="G30" s="234"/>
-      <c r="H30" s="234"/>
-      <c r="I30" s="234"/>
-      <c r="J30" s="234"/>
-      <c r="K30" s="235"/>
-      <c r="L30" s="233"/>
-      <c r="M30" s="234"/>
-      <c r="N30" s="234"/>
-      <c r="O30" s="234"/>
-      <c r="P30" s="234"/>
-      <c r="Q30" s="234"/>
-      <c r="R30" s="234"/>
-      <c r="S30" s="234"/>
-      <c r="T30" s="234"/>
-      <c r="U30" s="235"/>
+      <c r="A30" s="147"/>
+      <c r="B30" s="147"/>
+      <c r="C30" s="148"/>
+      <c r="D30" s="151"/>
+      <c r="E30" s="152"/>
+      <c r="F30" s="162"/>
+      <c r="G30" s="163"/>
+      <c r="H30" s="163"/>
+      <c r="I30" s="163"/>
+      <c r="J30" s="163"/>
+      <c r="K30" s="164"/>
+      <c r="L30" s="162"/>
+      <c r="M30" s="163"/>
+      <c r="N30" s="163"/>
+      <c r="O30" s="163"/>
+      <c r="P30" s="163"/>
+      <c r="Q30" s="163"/>
+      <c r="R30" s="163"/>
+      <c r="S30" s="163"/>
+      <c r="T30" s="163"/>
+      <c r="U30" s="164"/>
     </row>
     <row r="31" spans="1:25" ht="24.75" customHeight="1">
-      <c r="A31" s="218"/>
-      <c r="B31" s="218"/>
-      <c r="C31" s="219"/>
-      <c r="D31" s="222"/>
-      <c r="E31" s="223"/>
-      <c r="F31" s="233"/>
-      <c r="G31" s="234"/>
-      <c r="H31" s="234"/>
-      <c r="I31" s="234"/>
-      <c r="J31" s="234"/>
-      <c r="K31" s="235"/>
-      <c r="L31" s="233"/>
-      <c r="M31" s="234"/>
-      <c r="N31" s="234"/>
-      <c r="O31" s="234"/>
-      <c r="P31" s="234"/>
-      <c r="Q31" s="234"/>
-      <c r="R31" s="234"/>
-      <c r="S31" s="234"/>
-      <c r="T31" s="234"/>
-      <c r="U31" s="235"/>
+      <c r="A31" s="147"/>
+      <c r="B31" s="147"/>
+      <c r="C31" s="148"/>
+      <c r="D31" s="151"/>
+      <c r="E31" s="152"/>
+      <c r="F31" s="162"/>
+      <c r="G31" s="163"/>
+      <c r="H31" s="163"/>
+      <c r="I31" s="163"/>
+      <c r="J31" s="163"/>
+      <c r="K31" s="164"/>
+      <c r="L31" s="162"/>
+      <c r="M31" s="163"/>
+      <c r="N31" s="163"/>
+      <c r="O31" s="163"/>
+      <c r="P31" s="163"/>
+      <c r="Q31" s="163"/>
+      <c r="R31" s="163"/>
+      <c r="S31" s="163"/>
+      <c r="T31" s="163"/>
+      <c r="U31" s="164"/>
     </row>
     <row r="32" spans="1:25" ht="24.75" customHeight="1">
-      <c r="A32" s="218"/>
-      <c r="B32" s="218"/>
-      <c r="C32" s="219"/>
-      <c r="D32" s="222"/>
-      <c r="E32" s="223"/>
-      <c r="F32" s="233"/>
-      <c r="G32" s="234"/>
-      <c r="H32" s="234"/>
-      <c r="I32" s="234"/>
-      <c r="J32" s="234"/>
-      <c r="K32" s="235"/>
-      <c r="L32" s="233"/>
-      <c r="M32" s="234"/>
-      <c r="N32" s="234"/>
-      <c r="O32" s="234"/>
-      <c r="P32" s="234"/>
-      <c r="Q32" s="234"/>
-      <c r="R32" s="234"/>
-      <c r="S32" s="234"/>
-      <c r="T32" s="234"/>
-      <c r="U32" s="235"/>
+      <c r="A32" s="147"/>
+      <c r="B32" s="147"/>
+      <c r="C32" s="148"/>
+      <c r="D32" s="151"/>
+      <c r="E32" s="152"/>
+      <c r="F32" s="162"/>
+      <c r="G32" s="163"/>
+      <c r="H32" s="163"/>
+      <c r="I32" s="163"/>
+      <c r="J32" s="163"/>
+      <c r="K32" s="164"/>
+      <c r="L32" s="162"/>
+      <c r="M32" s="163"/>
+      <c r="N32" s="163"/>
+      <c r="O32" s="163"/>
+      <c r="P32" s="163"/>
+      <c r="Q32" s="163"/>
+      <c r="R32" s="163"/>
+      <c r="S32" s="163"/>
+      <c r="T32" s="163"/>
+      <c r="U32" s="164"/>
     </row>
     <row r="33" spans="1:21" ht="28.5" customHeight="1">
-      <c r="A33" s="218"/>
-      <c r="B33" s="218"/>
-      <c r="C33" s="219"/>
-      <c r="D33" s="222"/>
-      <c r="E33" s="223"/>
-      <c r="F33" s="233"/>
-      <c r="G33" s="234"/>
-      <c r="H33" s="234"/>
-      <c r="I33" s="234"/>
-      <c r="J33" s="234"/>
-      <c r="K33" s="235"/>
-      <c r="L33" s="233"/>
-      <c r="M33" s="234"/>
-      <c r="N33" s="234"/>
-      <c r="O33" s="234"/>
-      <c r="P33" s="234"/>
-      <c r="Q33" s="234"/>
-      <c r="R33" s="234"/>
-      <c r="S33" s="234"/>
-      <c r="T33" s="234"/>
-      <c r="U33" s="235"/>
+      <c r="A33" s="147"/>
+      <c r="B33" s="147"/>
+      <c r="C33" s="148"/>
+      <c r="D33" s="151"/>
+      <c r="E33" s="152"/>
+      <c r="F33" s="162"/>
+      <c r="G33" s="163"/>
+      <c r="H33" s="163"/>
+      <c r="I33" s="163"/>
+      <c r="J33" s="163"/>
+      <c r="K33" s="164"/>
+      <c r="L33" s="162"/>
+      <c r="M33" s="163"/>
+      <c r="N33" s="163"/>
+      <c r="O33" s="163"/>
+      <c r="P33" s="163"/>
+      <c r="Q33" s="163"/>
+      <c r="R33" s="163"/>
+      <c r="S33" s="163"/>
+      <c r="T33" s="163"/>
+      <c r="U33" s="164"/>
     </row>
     <row r="34" spans="1:21" ht="24.75" customHeight="1">
-      <c r="A34" s="218"/>
-      <c r="B34" s="218"/>
-      <c r="C34" s="219"/>
-      <c r="D34" s="222"/>
-      <c r="E34" s="223"/>
-      <c r="F34" s="233"/>
-      <c r="G34" s="234"/>
-      <c r="H34" s="234"/>
-      <c r="I34" s="234"/>
-      <c r="J34" s="234"/>
-      <c r="K34" s="235"/>
-      <c r="L34" s="233"/>
-      <c r="M34" s="234"/>
-      <c r="N34" s="234"/>
-      <c r="O34" s="234"/>
-      <c r="P34" s="234"/>
-      <c r="Q34" s="234"/>
-      <c r="R34" s="234"/>
-      <c r="S34" s="234"/>
-      <c r="T34" s="234"/>
-      <c r="U34" s="235"/>
+      <c r="A34" s="147"/>
+      <c r="B34" s="147"/>
+      <c r="C34" s="148"/>
+      <c r="D34" s="151"/>
+      <c r="E34" s="152"/>
+      <c r="F34" s="162"/>
+      <c r="G34" s="163"/>
+      <c r="H34" s="163"/>
+      <c r="I34" s="163"/>
+      <c r="J34" s="163"/>
+      <c r="K34" s="164"/>
+      <c r="L34" s="162"/>
+      <c r="M34" s="163"/>
+      <c r="N34" s="163"/>
+      <c r="O34" s="163"/>
+      <c r="P34" s="163"/>
+      <c r="Q34" s="163"/>
+      <c r="R34" s="163"/>
+      <c r="S34" s="163"/>
+      <c r="T34" s="163"/>
+      <c r="U34" s="164"/>
     </row>
     <row r="35" spans="1:21" ht="24.75" customHeight="1">
-      <c r="A35" s="218"/>
-      <c r="B35" s="218"/>
-      <c r="C35" s="219"/>
-      <c r="D35" s="222"/>
-      <c r="E35" s="223"/>
-      <c r="F35" s="233"/>
-      <c r="G35" s="234"/>
-      <c r="H35" s="234"/>
-      <c r="I35" s="234"/>
-      <c r="J35" s="234"/>
-      <c r="K35" s="235"/>
-      <c r="L35" s="233"/>
-      <c r="M35" s="234"/>
-      <c r="N35" s="234"/>
-      <c r="O35" s="234"/>
-      <c r="P35" s="234"/>
-      <c r="Q35" s="234"/>
-      <c r="R35" s="234"/>
-      <c r="S35" s="234"/>
-      <c r="T35" s="234"/>
-      <c r="U35" s="235"/>
+      <c r="A35" s="147"/>
+      <c r="B35" s="147"/>
+      <c r="C35" s="148"/>
+      <c r="D35" s="151"/>
+      <c r="E35" s="152"/>
+      <c r="F35" s="162"/>
+      <c r="G35" s="163"/>
+      <c r="H35" s="163"/>
+      <c r="I35" s="163"/>
+      <c r="J35" s="163"/>
+      <c r="K35" s="164"/>
+      <c r="L35" s="162"/>
+      <c r="M35" s="163"/>
+      <c r="N35" s="163"/>
+      <c r="O35" s="163"/>
+      <c r="P35" s="163"/>
+      <c r="Q35" s="163"/>
+      <c r="R35" s="163"/>
+      <c r="S35" s="163"/>
+      <c r="T35" s="163"/>
+      <c r="U35" s="164"/>
     </row>
     <row r="36" spans="1:21" ht="30.75" customHeight="1">
-      <c r="A36" s="254"/>
-      <c r="B36" s="218"/>
-      <c r="C36" s="219"/>
-      <c r="D36" s="224"/>
-      <c r="E36" s="225"/>
-      <c r="F36" s="236"/>
-      <c r="G36" s="237"/>
-      <c r="H36" s="237"/>
-      <c r="I36" s="237"/>
-      <c r="J36" s="237"/>
-      <c r="K36" s="238"/>
-      <c r="L36" s="236"/>
-      <c r="M36" s="237"/>
-      <c r="N36" s="237"/>
-      <c r="O36" s="237"/>
-      <c r="P36" s="237"/>
-      <c r="Q36" s="237"/>
-      <c r="R36" s="237"/>
-      <c r="S36" s="237"/>
-      <c r="T36" s="237"/>
-      <c r="U36" s="238"/>
+      <c r="A36" s="187"/>
+      <c r="B36" s="147"/>
+      <c r="C36" s="148"/>
+      <c r="D36" s="153"/>
+      <c r="E36" s="154"/>
+      <c r="F36" s="165"/>
+      <c r="G36" s="166"/>
+      <c r="H36" s="166"/>
+      <c r="I36" s="166"/>
+      <c r="J36" s="166"/>
+      <c r="K36" s="167"/>
+      <c r="L36" s="165"/>
+      <c r="M36" s="166"/>
+      <c r="N36" s="166"/>
+      <c r="O36" s="166"/>
+      <c r="P36" s="166"/>
+      <c r="Q36" s="166"/>
+      <c r="R36" s="166"/>
+      <c r="S36" s="166"/>
+      <c r="T36" s="166"/>
+      <c r="U36" s="167"/>
     </row>
     <row r="37" spans="1:21" ht="39" customHeight="1">
       <c r="A37" s="75">
         <f>D11</f>
         <v>0</v>
       </c>
-      <c r="B37" s="164">
+      <c r="B37" s="176">
         <f>D12</f>
         <v>0</v>
       </c>
-      <c r="C37" s="165"/>
-      <c r="D37" s="164"/>
-      <c r="E37" s="165"/>
-      <c r="F37" s="166"/>
-      <c r="G37" s="167"/>
-      <c r="H37" s="167"/>
-      <c r="I37" s="167"/>
-      <c r="J37" s="167"/>
-      <c r="K37" s="168"/>
-      <c r="L37" s="169"/>
-      <c r="M37" s="170"/>
-      <c r="N37" s="170"/>
-      <c r="O37" s="170"/>
-      <c r="P37" s="171"/>
-      <c r="Q37" s="172"/>
-      <c r="R37" s="172"/>
-      <c r="S37" s="172"/>
-      <c r="T37" s="172"/>
-      <c r="U37" s="173"/>
+      <c r="C37" s="219"/>
+      <c r="D37" s="176"/>
+      <c r="E37" s="219"/>
+      <c r="F37" s="220"/>
+      <c r="G37" s="221"/>
+      <c r="H37" s="221"/>
+      <c r="I37" s="221"/>
+      <c r="J37" s="221"/>
+      <c r="K37" s="222"/>
+      <c r="L37" s="223"/>
+      <c r="M37" s="224"/>
+      <c r="N37" s="224"/>
+      <c r="O37" s="224"/>
+      <c r="P37" s="225"/>
+      <c r="Q37" s="226"/>
+      <c r="R37" s="226"/>
+      <c r="S37" s="226"/>
+      <c r="T37" s="226"/>
+      <c r="U37" s="227"/>
     </row>
     <row r="38" spans="1:21" ht="14.25" customHeight="1">
-      <c r="A38" s="164"/>
-      <c r="B38" s="247"/>
-      <c r="C38" s="247"/>
-      <c r="D38" s="248"/>
-      <c r="E38" s="248"/>
-      <c r="F38" s="247"/>
-      <c r="G38" s="247"/>
-      <c r="H38" s="247"/>
-      <c r="I38" s="247"/>
-      <c r="J38" s="247"/>
-      <c r="K38" s="247"/>
-      <c r="L38" s="247"/>
-      <c r="M38" s="247"/>
-      <c r="N38" s="247"/>
-      <c r="O38" s="247"/>
-      <c r="P38" s="247"/>
-      <c r="Q38" s="247"/>
-      <c r="R38" s="247"/>
-      <c r="S38" s="249"/>
+      <c r="A38" s="176"/>
+      <c r="B38" s="177"/>
+      <c r="C38" s="177"/>
+      <c r="D38" s="178"/>
+      <c r="E38" s="178"/>
+      <c r="F38" s="177"/>
+      <c r="G38" s="177"/>
+      <c r="H38" s="177"/>
+      <c r="I38" s="177"/>
+      <c r="J38" s="177"/>
+      <c r="K38" s="177"/>
+      <c r="L38" s="177"/>
+      <c r="M38" s="177"/>
+      <c r="N38" s="177"/>
+      <c r="O38" s="177"/>
+      <c r="P38" s="177"/>
+      <c r="Q38" s="177"/>
+      <c r="R38" s="177"/>
+      <c r="S38" s="179"/>
       <c r="T38" s="25"/>
       <c r="U38" s="25"/>
     </row>
     <row r="39" spans="1:21">
-      <c r="A39" s="161" t="s">
+      <c r="A39" s="180" t="s">
         <v>34</v>
       </c>
-      <c r="B39" s="250"/>
-      <c r="C39" s="251" t="s">
+      <c r="B39" s="181"/>
+      <c r="C39" s="182" t="s">
         <v>35</v>
       </c>
-      <c r="D39" s="252"/>
-      <c r="E39" s="252"/>
-      <c r="F39" s="252"/>
-      <c r="G39" s="252"/>
-      <c r="H39" s="252"/>
-      <c r="I39" s="252"/>
-      <c r="J39" s="252"/>
-      <c r="K39" s="253"/>
-      <c r="L39" s="162" t="s">
+      <c r="D39" s="183"/>
+      <c r="E39" s="183"/>
+      <c r="F39" s="183"/>
+      <c r="G39" s="183"/>
+      <c r="H39" s="183"/>
+      <c r="I39" s="183"/>
+      <c r="J39" s="183"/>
+      <c r="K39" s="184"/>
+      <c r="L39" s="185" t="s">
         <v>36</v>
       </c>
-      <c r="M39" s="162"/>
-      <c r="N39" s="162"/>
-      <c r="O39" s="162"/>
-      <c r="P39" s="163"/>
-      <c r="Q39" s="161" t="s">
+      <c r="M39" s="185"/>
+      <c r="N39" s="185"/>
+      <c r="O39" s="185"/>
+      <c r="P39" s="186"/>
+      <c r="Q39" s="180" t="s">
         <v>37</v>
       </c>
-      <c r="R39" s="162"/>
-      <c r="S39" s="163"/>
-      <c r="T39" s="174" t="s">
+      <c r="R39" s="185"/>
+      <c r="S39" s="186"/>
+      <c r="T39" s="228" t="s">
         <v>38</v>
       </c>
-      <c r="U39" s="175"/>
+      <c r="U39" s="229"/>
     </row>
     <row r="40" spans="1:21">
-      <c r="A40" s="239" t="s">
+      <c r="A40" s="168" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="240"/>
-      <c r="C40" s="239" t="s">
+      <c r="B40" s="169"/>
+      <c r="C40" s="168" t="s">
         <v>40</v>
       </c>
-      <c r="D40" s="240"/>
-      <c r="E40" s="240"/>
-      <c r="F40" s="240"/>
-      <c r="G40" s="240"/>
-      <c r="H40" s="240"/>
-      <c r="I40" s="240"/>
-      <c r="J40" s="240"/>
-      <c r="K40" s="241"/>
-      <c r="L40" s="240" t="s">
+      <c r="D40" s="169"/>
+      <c r="E40" s="169"/>
+      <c r="F40" s="169"/>
+      <c r="G40" s="169"/>
+      <c r="H40" s="169"/>
+      <c r="I40" s="169"/>
+      <c r="J40" s="169"/>
+      <c r="K40" s="170"/>
+      <c r="L40" s="169" t="s">
         <v>41</v>
       </c>
-      <c r="M40" s="240"/>
-      <c r="N40" s="240"/>
-      <c r="O40" s="240"/>
-      <c r="P40" s="241"/>
-      <c r="Q40" s="242" t="s">
+      <c r="M40" s="169"/>
+      <c r="N40" s="169"/>
+      <c r="O40" s="169"/>
+      <c r="P40" s="170"/>
+      <c r="Q40" s="171" t="s">
         <v>42</v>
       </c>
-      <c r="R40" s="243"/>
-      <c r="S40" s="244"/>
-      <c r="T40" s="176"/>
-      <c r="U40" s="177"/>
+      <c r="R40" s="172"/>
+      <c r="S40" s="173"/>
+      <c r="T40" s="230"/>
+      <c r="U40" s="231"/>
     </row>
     <row r="41" spans="1:21">
       <c r="A41" s="76"/>
@@ -5461,8 +5462,8 @@
       <c r="Q41" s="136"/>
       <c r="R41" s="79"/>
       <c r="S41" s="137"/>
-      <c r="T41" s="214"/>
-      <c r="U41" s="215"/>
+      <c r="T41" s="143"/>
+      <c r="U41" s="144"/>
     </row>
     <row r="42" spans="1:21">
       <c r="A42" s="76"/>
@@ -5484,8 +5485,8 @@
       <c r="Q42" s="76"/>
       <c r="R42" s="77"/>
       <c r="S42" s="138"/>
-      <c r="T42" s="214"/>
-      <c r="U42" s="215"/>
+      <c r="T42" s="143"/>
+      <c r="U42" s="144"/>
     </row>
     <row r="43" spans="1:21">
       <c r="A43" s="76"/>
@@ -5507,8 +5508,8 @@
       <c r="Q43" s="76"/>
       <c r="R43" s="77"/>
       <c r="S43" s="138"/>
-      <c r="T43" s="214"/>
-      <c r="U43" s="215"/>
+      <c r="T43" s="143"/>
+      <c r="U43" s="144"/>
     </row>
     <row r="44" spans="1:21">
       <c r="A44" s="76"/>
@@ -5530,8 +5531,8 @@
       <c r="Q44" s="76"/>
       <c r="R44" s="77"/>
       <c r="S44" s="138"/>
-      <c r="T44" s="214"/>
-      <c r="U44" s="215"/>
+      <c r="T44" s="143"/>
+      <c r="U44" s="144"/>
     </row>
     <row r="45" spans="1:21">
       <c r="A45" s="76"/>
@@ -5553,8 +5554,8 @@
       <c r="Q45" s="76"/>
       <c r="R45" s="77"/>
       <c r="S45" s="138"/>
-      <c r="T45" s="214"/>
-      <c r="U45" s="215"/>
+      <c r="T45" s="143"/>
+      <c r="U45" s="144"/>
     </row>
     <row r="46" spans="1:21">
       <c r="A46" s="76"/>
@@ -5576,8 +5577,8 @@
       <c r="Q46" s="139"/>
       <c r="R46" s="140"/>
       <c r="S46" s="138"/>
-      <c r="T46" s="214"/>
-      <c r="U46" s="215"/>
+      <c r="T46" s="143"/>
+      <c r="U46" s="144"/>
     </row>
     <row r="47" spans="1:21">
       <c r="A47" s="76"/>
@@ -5599,8 +5600,8 @@
       <c r="Q47" s="139"/>
       <c r="R47" s="140"/>
       <c r="S47" s="138"/>
-      <c r="T47" s="214"/>
-      <c r="U47" s="215"/>
+      <c r="T47" s="143"/>
+      <c r="U47" s="144"/>
     </row>
     <row r="48" spans="1:21" ht="18.75">
       <c r="A48" s="76"/>
@@ -5622,8 +5623,8 @@
       <c r="Q48" s="139"/>
       <c r="R48" s="140"/>
       <c r="S48" s="138"/>
-      <c r="T48" s="214"/>
-      <c r="U48" s="215"/>
+      <c r="T48" s="143"/>
+      <c r="U48" s="144"/>
     </row>
     <row r="49" spans="1:21">
       <c r="A49" s="76"/>
@@ -5645,8 +5646,8 @@
       <c r="Q49" s="139"/>
       <c r="R49" s="140"/>
       <c r="S49" s="138"/>
-      <c r="T49" s="214"/>
-      <c r="U49" s="215"/>
+      <c r="T49" s="143"/>
+      <c r="U49" s="144"/>
     </row>
     <row r="50" spans="1:21" ht="18.75">
       <c r="A50" s="76"/>
@@ -5660,18 +5661,18 @@
       <c r="I50" s="103"/>
       <c r="J50" s="103"/>
       <c r="K50" s="104"/>
-      <c r="L50" s="245" t="s">
+      <c r="L50" s="174" t="s">
         <v>43</v>
       </c>
-      <c r="M50" s="245"/>
-      <c r="N50" s="245"/>
-      <c r="O50" s="245"/>
-      <c r="P50" s="246"/>
+      <c r="M50" s="174"/>
+      <c r="N50" s="174"/>
+      <c r="O50" s="174"/>
+      <c r="P50" s="175"/>
       <c r="Q50" s="139"/>
       <c r="R50" s="140"/>
       <c r="S50" s="138"/>
-      <c r="T50" s="214"/>
-      <c r="U50" s="215"/>
+      <c r="T50" s="143"/>
+      <c r="U50" s="144"/>
     </row>
     <row r="51" spans="1:21">
       <c r="A51" s="76"/>
@@ -5693,8 +5694,8 @@
       <c r="Q51" s="139"/>
       <c r="R51" s="140"/>
       <c r="S51" s="138"/>
-      <c r="T51" s="214"/>
-      <c r="U51" s="215"/>
+      <c r="T51" s="143"/>
+      <c r="U51" s="144"/>
     </row>
     <row r="52" spans="1:21">
       <c r="A52" s="76"/>
@@ -5716,8 +5717,8 @@
       <c r="Q52" s="139"/>
       <c r="R52" s="140"/>
       <c r="S52" s="138"/>
-      <c r="T52" s="214"/>
-      <c r="U52" s="215"/>
+      <c r="T52" s="143"/>
+      <c r="U52" s="144"/>
     </row>
     <row r="53" spans="1:21">
       <c r="A53" s="86"/>
@@ -5739,11 +5740,61 @@
       <c r="Q53" s="141"/>
       <c r="R53" s="111"/>
       <c r="S53" s="142"/>
-      <c r="T53" s="214"/>
-      <c r="U53" s="215"/>
+      <c r="T53" s="143"/>
+      <c r="U53" s="144"/>
     </row>
   </sheetData>
   <mergeCells count="66">
+    <mergeCell ref="E4:K4"/>
+    <mergeCell ref="N4:U4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="N5:U5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="N6:S6"/>
+    <mergeCell ref="E5:K5"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="N1:U1"/>
+    <mergeCell ref="E2:K2"/>
+    <mergeCell ref="N2:U2"/>
+    <mergeCell ref="E3:K3"/>
+    <mergeCell ref="N3:U3"/>
+    <mergeCell ref="A27:U27"/>
+    <mergeCell ref="S8:S9"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="Q39:S39"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="F37:K37"/>
+    <mergeCell ref="L37:P37"/>
+    <mergeCell ref="Q37:U37"/>
+    <mergeCell ref="T39:U40"/>
+    <mergeCell ref="B24:D25"/>
+    <mergeCell ref="B21:D22"/>
+    <mergeCell ref="B19:D20"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="P9:P10"/>
+    <mergeCell ref="Q9:Q10"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:K28"/>
+    <mergeCell ref="L28:U28"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="R8:R10"/>
+    <mergeCell ref="F8:Q8"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
     <mergeCell ref="T41:U53"/>
     <mergeCell ref="B29:C36"/>
     <mergeCell ref="D29:E36"/>
@@ -5760,56 +5811,6 @@
     <mergeCell ref="C39:K39"/>
     <mergeCell ref="L39:P39"/>
     <mergeCell ref="A29:A36"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:K28"/>
-    <mergeCell ref="L28:U28"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="R8:R10"/>
-    <mergeCell ref="F8:Q8"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="A27:U27"/>
-    <mergeCell ref="S8:S9"/>
-    <mergeCell ref="T8:T9"/>
-    <mergeCell ref="Q39:S39"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="F37:K37"/>
-    <mergeCell ref="L37:P37"/>
-    <mergeCell ref="Q37:U37"/>
-    <mergeCell ref="T39:U40"/>
-    <mergeCell ref="B24:D25"/>
-    <mergeCell ref="B21:D22"/>
-    <mergeCell ref="B19:D20"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="P9:P10"/>
-    <mergeCell ref="Q9:Q10"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="N1:U1"/>
-    <mergeCell ref="E2:K2"/>
-    <mergeCell ref="N2:U2"/>
-    <mergeCell ref="E3:K3"/>
-    <mergeCell ref="N3:U3"/>
-    <mergeCell ref="E4:K4"/>
-    <mergeCell ref="N4:U4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="N5:U5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="N6:S6"/>
-    <mergeCell ref="E5:K5"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.11811023622047245" bottom="0.11811023622047245" header="0.11811023622047245" footer="0.11811023622047245"/>

</xml_diff>